<commit_message>
GL-4 DD_GINI_P2 small change to keep consistent with P1
</commit_message>
<xml_diff>
--- a/rmonize/data_dictionary/DD_GINI_P2.xlsx
+++ b/rmonize/data_dictionary/DD_GINI_P2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD21E3E3-026B-4F0D-9D04-99753C54CA03}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87F842C-E164-41D5-838E-1D84B1162DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22290" windowHeight="12000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="189">
   <si>
     <t>index</t>
   </si>
@@ -590,6 +590,9 @@
   </si>
   <si>
     <t>Glycemic Load calculated from FFQ data</t>
+  </si>
+  <si>
+    <t>Hochschule/Fachhochschule/Universität</t>
   </si>
 </sst>
 </file>
@@ -748,9 +751,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -788,7 +791,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -894,7 +897,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1036,7 +1039,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2494,7 +2497,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>111</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2919,6 +2922,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B1DC67C611DD5E4D81775F9F3E26A7B2" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7f379a5812b480a74f9d031be5f88a83">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xmlns:ns3="12535b08-222e-45d2-b6db-15019f1afee6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbce1e37d7de67e1c835013ca0ee7a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
@@ -3159,18 +3174,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C05FF1B-7508-40EF-8319-E993EA07F007}">
   <ds:schemaRefs>
@@ -3180,6 +3183,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D9CBEFE-8C4C-4054-8E02-CA457E93B4C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
+    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{916FD215-94E3-49D7-AFA2-532F4DA2AAAC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3196,15 +3210,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D9CBEFE-8C4C-4054-8E02-CA457E93B4C8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
-    <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>